<commit_message>
feat: backfill Anthropic, OpenAI and xAI — universe complete
Finishes the funding-history backfill. The store now holds 239 facts, up
from 130 at the start of the day. Twelve of thirteen companies carry a
dated valuation ladder; CoreWeave is the exception because it listed
publicly in 2025, so its history lives in filings rather than private
deal records.

Anthropic: 6 marks, 2024-07 to 2026-05.
OpenAI: 6 marks, 2024-01 to 2026-03.
xAI: 5 marks, 2024-05 to 2026-02.

Models rebuilt against the fuller store. Four remain mechanically sound;
none is research-grade. Revenue is still the binding constraint — the
backfill supplies cap tables, not income statements, which is the case
recommendation 1 makes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WBFso58BAR4Z1QWa1Tfo4w
</commit_message>
<xml_diff>
--- a/companies/anthropic/financials/anthropic_model_2026-08-14.xlsx
+++ b/companies/anthropic/financials/anthropic_model_2026-08-14.xlsx
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J24"/>
+  <dimension ref="B2:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1605,16 +1605,16 @@
     <row r="10">
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>Total raised (equity and debt)</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr"/>
       <c r="D10" s="30" t="n">
-        <v>161.3</v>
+        <v>21</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1624,23 +1624,23 @@
       </c>
       <c r="J10" s="29" t="inlineStr">
         <is>
-          <t>PitchBook total raised $161.254B, confirmed live</t>
+          <t>PitchBook deal 265998-97T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>Equity raised</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr"/>
       <c r="D11" s="30" t="n">
-        <v>124.3</v>
+        <v>54</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2024-11-22</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1650,23 +1650,23 @@
       </c>
       <c r="J11" s="29" t="inlineStr">
         <is>
-          <t>canonical decomposition: excludes $34.5B chip bonds + $2.5B revolver</t>
+          <t>PitchBook deal 276864-04T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>Debt raised</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr"/>
       <c r="D12" s="30" t="n">
-        <v>37</v>
+        <v>61.5</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2025-03-03</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1676,23 +1676,23 @@
       </c>
       <c r="J12" s="29" t="inlineStr">
         <is>
-          <t>PB 334763-02T ($34.5B tranched chip bonds) + 295197-04T ($2.5B revolver)</t>
+          <t>PitchBook deal 281518-66T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>Annualised revenue</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr"/>
       <c r="D13" s="30" t="n">
-        <v>47</v>
+        <v>183</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2025-09-02</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -1702,23 +1702,23 @@
       </c>
       <c r="J13" s="29" t="inlineStr">
         <is>
-          <t>company-announced run-rate (gross basis)</t>
+          <t>PitchBook deal 287700-58T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>Fy2025 revenue ($bn)</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr"/>
       <c r="D14" s="30" t="n">
-        <v>9</v>
+        <v>380</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
@@ -1728,25 +1728,23 @@
       </c>
       <c r="J14" s="29" t="inlineStr">
         <is>
-          <t>PitchBook financials</t>
+          <t>PitchBook deal 313890-49T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>Note on the PitchBook revenue field</t>
+          <t>Valuation history</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr"/>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>PB revenue field $55B TTM 4Q2027 (period end 2027-12-31) = f</t>
-        </is>
+      <c r="D15" s="30" t="n">
+        <v>965</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -1756,51 +1754,49 @@
       </c>
       <c r="J15" s="29" t="inlineStr">
         <is>
-          <t>canonical refresh, July 16, 2026</t>
+          <t>PitchBook deal 329489-02T (Later Stage VC)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>First operating profit</t>
+          <t>Total raised (equity and debt)</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr"/>
-      <c r="D16" s="15" t="inlineStr">
-        <is>
-          <t>~$559M expected Q2 2026</t>
-        </is>
+      <c r="D16" s="30" t="n">
+        <v>161.3</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="J16" s="29" t="inlineStr">
         <is>
-          <t>press reports</t>
+          <t>PitchBook total raised $161.254B, confirmed live</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>Employees</t>
+          <t>Equity raised</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr"/>
       <c r="D17" s="30" t="n">
-        <v>5000</v>
+        <v>124.3</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -1810,25 +1806,23 @@
       </c>
       <c r="J17" s="29" t="inlineStr">
         <is>
-          <t>PitchBook</t>
+          <t>canonical decomposition: excludes $34.5B chip bonds + $2.5B revolver</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>Net revenue retention</t>
+          <t>Debt raised</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr"/>
-      <c r="D18" s="15" t="inlineStr">
-        <is>
-          <t>140%+</t>
-        </is>
+      <c r="D18" s="30" t="n">
+        <v>37</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
@@ -1838,25 +1832,25 @@
       </c>
       <c r="J18" s="29" t="inlineStr">
         <is>
-          <t>company-announced</t>
+          <t>PB 334763-02T ($34.5B tranched chip bonds) + 295197-04T ($2.5B revolver)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Business customers</t>
+          <t>Last completed round</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr"/>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>300K+</t>
+          <t>Debt - General $34500M (round n/a)</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -1866,25 +1860,23 @@
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>company-announced</t>
+          <t>PitchBook deal 334763-02T</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Acv 1m plus</t>
+          <t>Raised to date ($bn)</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr"/>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>1,000+</t>
-        </is>
+      <c r="D20" s="30" t="n">
+        <v>161.254</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
@@ -1894,23 +1886,25 @@
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>company-announced</t>
+          <t>PitchBook Raised to Date, deal 334763-02T</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>Claude code arr ($bn)</t>
+          <t>Deal history</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr"/>
-      <c r="D21" s="30" t="n">
-        <v>2.5</v>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>2024-05-31 Secondary Transaction - Private $1,320M; 2024-07-</t>
+        </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
@@ -1920,25 +1914,23 @@
       </c>
       <c r="J21" s="29" t="inlineStr">
         <is>
-          <t>company-announced</t>
+          <t>PitchBook deal history</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>IPO filing status</t>
+          <t>Annualised revenue</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr"/>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>Confidential S-1 filed Jun 1, 2026</t>
-        </is>
+      <c r="D22" s="30" t="n">
+        <v>47</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
@@ -1948,21 +1940,19 @@
       </c>
       <c r="J22" s="29" t="inlineStr">
         <is>
-          <t>press + PitchBook</t>
+          <t>company-announced run-rate (gross basis)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>Expected IPO window</t>
+          <t>Fy2025 revenue ($bn)</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr"/>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>October 2026 expected (PitchBook financing note, refreshed J</t>
-        </is>
+      <c r="D23" s="30" t="n">
+        <v>9</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1976,31 +1966,279 @@
       </c>
       <c r="J23" s="29" t="inlineStr">
         <is>
-          <t>PitchBook</t>
+          <t>PitchBook financials</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="17" t="inlineStr">
         <is>
+          <t>Note on the PitchBook revenue field</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>PB revenue field $55B TTM 4Q2027 (period end 2027-12-31) = f</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J24" s="29" t="inlineStr">
+        <is>
+          <t>canonical refresh, July 16, 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>First operating profit</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr"/>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>~$559M expected Q2 2026</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="J25" s="29" t="inlineStr">
+        <is>
+          <t>press reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Employees</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr"/>
+      <c r="D26" s="30" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J26" s="29" t="inlineStr">
+        <is>
+          <t>PitchBook</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>Net revenue retention</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr"/>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>140%+</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J27" s="29" t="inlineStr">
+        <is>
+          <t>company-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Business customers</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr"/>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>300K+</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J28" s="29" t="inlineStr">
+        <is>
+          <t>company-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Acv 1m plus</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr"/>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>1,000+</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J29" s="29" t="inlineStr">
+        <is>
+          <t>company-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>Claude code arr ($bn)</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr"/>
+      <c r="D30" s="30" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J30" s="29" t="inlineStr">
+        <is>
+          <t>company-announced</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>IPO filing status</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr"/>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>Confidential S-1 filed Jun 1, 2026</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J31" s="29" t="inlineStr">
+        <is>
+          <t>press + PitchBook</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Expected IPO window</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr"/>
+      <c r="D32" s="15" t="inlineStr">
+        <is>
+          <t>October 2026 expected (PitchBook financing note, refreshed J</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="J32" s="29" t="inlineStr">
+        <is>
+          <t>PitchBook</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="17" t="inlineStr">
+        <is>
           <t>Quality score (composite)</t>
         </is>
       </c>
-      <c r="C24" s="17" t="inlineStr"/>
-      <c r="D24" s="30" t="n">
+      <c r="C33" s="17" t="inlineStr"/>
+      <c r="D33" s="30" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="F24" s="7" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>2026-05-27</t>
         </is>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>T2</t>
         </is>
       </c>
-      <c r="J24" s="29" t="inlineStr">
+      <c r="J33" s="29" t="inlineStr">
         <is>
           <t>internal AIBQ v3.0 (this desk)</t>
         </is>

</xml_diff>